<commit_message>
updated input data and subsequent analyses
</commit_message>
<xml_diff>
--- a/LOT2_samples.xlsx
+++ b/LOT2_samples.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valeriehofstetter/Desktop/LoT2_PAPER/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E291A4-0F4D-BA4C-8F92-C76D4B86EC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD45091-8E52-D040-B06D-9CA2B652D3F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="660" windowWidth="18360" windowHeight="20060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1620" yWindow="600" windowWidth="29400" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL isolates" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7648" uniqueCount="2004">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7648" uniqueCount="2007">
   <si>
     <t>Hofstetter-Code</t>
   </si>
@@ -9700,6 +9700,15 @@
   </si>
   <si>
     <t xml:space="preserve">Sordariomycetes sp. 5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">S5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">S10 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">S9 </t>
   </si>
 </sst>
 </file>
@@ -10004,7 +10013,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -10384,9 +10393,6 @@
     <xf numFmtId="0" fontId="5" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -10701,12 +10707,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{157218CF-639F-48E2-9064-BC6FA5AB1532}">
   <dimension ref="A1:H747"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="20.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" style="51" customWidth="1"/>
     <col min="2" max="2" width="8.1640625" style="20" customWidth="1"/>
     <col min="3" max="3" width="13" style="20" customWidth="1"/>
-    <col min="4" max="4" width="15" style="52" customWidth="1"/>
+    <col min="4" max="4" width="15" style="38" customWidth="1"/>
     <col min="5" max="5" width="15.33203125" style="20" customWidth="1"/>
     <col min="6" max="6" width="73.1640625" style="20" customWidth="1"/>
     <col min="7" max="7" width="60.6640625" style="20" customWidth="1"/>
@@ -10724,7 +10730,7 @@
       <c r="C1" s="126" t="s">
         <v>1885</v>
       </c>
-      <c r="D1" s="128" t="s">
+      <c r="D1" s="127" t="s">
         <v>1884</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -10748,7 +10754,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="39" t="s">
-        <v>274</v>
+        <v>2004</v>
       </c>
       <c r="E2" s="111">
         <v>575</v>
@@ -10771,7 +10777,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>274</v>
+        <v>2004</v>
       </c>
       <c r="E3" s="111">
         <v>576</v>
@@ -10840,9 +10846,9 @@
         <v>6</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>270</v>
-      </c>
-      <c r="D6" s="52" t="s">
+        <v>391</v>
+      </c>
+      <c r="D6" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E6" s="111">
@@ -10866,9 +10872,9 @@
         <v>6</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>274</v>
-      </c>
-      <c r="D7" s="52" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D7" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E7" s="18">
@@ -10894,7 +10900,7 @@
       <c r="C8" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D8" s="52" t="s">
+      <c r="D8" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E8" s="115">
@@ -11127,7 +11133,7 @@
       <c r="C18" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D18" s="52" t="s">
+      <c r="D18" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E18" s="18">
@@ -11153,7 +11159,7 @@
       <c r="C19" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D19" s="52" t="s">
+      <c r="D19" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E19" s="18">
@@ -11174,12 +11180,12 @@
         <v>267</v>
       </c>
       <c r="B20" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C20" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D20" s="52" t="s">
+      <c r="D20" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E20" s="18">
@@ -11249,7 +11255,7 @@
         <v>4</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>279</v>
+        <v>2005</v>
       </c>
       <c r="E23" s="111">
         <v>630</v>
@@ -11272,7 +11278,7 @@
         <v>5</v>
       </c>
       <c r="C24" s="113" t="s">
-        <v>278</v>
+        <v>2006</v>
       </c>
       <c r="E24" s="111">
         <v>614</v>
@@ -11294,7 +11300,7 @@
       <c r="B25" s="39">
         <v>5</v>
       </c>
-      <c r="C25" s="130" t="s">
+      <c r="C25" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E25" s="18">
@@ -11317,7 +11323,7 @@
       <c r="B26" s="39">
         <v>5</v>
       </c>
-      <c r="C26" s="130" t="s">
+      <c r="C26" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E26" s="18">
@@ -11340,7 +11346,7 @@
       <c r="B27" s="39">
         <v>4</v>
       </c>
-      <c r="C27" s="130" t="s">
+      <c r="C27" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E27" s="18">
@@ -11363,7 +11369,7 @@
       <c r="B28" s="39">
         <v>3</v>
       </c>
-      <c r="C28" s="130" t="s">
+      <c r="C28" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E28" s="18">
@@ -11386,7 +11392,7 @@
       <c r="B29" s="39">
         <v>3</v>
       </c>
-      <c r="C29" s="130" t="s">
+      <c r="C29" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E29" s="18">
@@ -11409,7 +11415,7 @@
       <c r="B30" s="39">
         <v>2</v>
       </c>
-      <c r="C30" s="130" t="s">
+      <c r="C30" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E30" s="18">
@@ -11432,7 +11438,7 @@
       <c r="B31" s="39">
         <v>2</v>
       </c>
-      <c r="C31" s="130" t="s">
+      <c r="C31" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E31" s="18">
@@ -11455,7 +11461,7 @@
       <c r="B32" s="39">
         <v>4</v>
       </c>
-      <c r="C32" s="130" t="s">
+      <c r="C32" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E32" s="111">
@@ -11478,7 +11484,7 @@
       <c r="B33" s="39">
         <v>4</v>
       </c>
-      <c r="C33" s="130" t="s">
+      <c r="C33" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E33" s="18">
@@ -11501,7 +11507,7 @@
       <c r="B34" s="39">
         <v>5</v>
       </c>
-      <c r="C34" s="130" t="s">
+      <c r="C34" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E34" s="111">
@@ -11524,7 +11530,7 @@
       <c r="B35" s="39">
         <v>3</v>
       </c>
-      <c r="C35" s="130" t="s">
+      <c r="C35" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E35" s="18">
@@ -11547,7 +11553,7 @@
       <c r="B36" s="39">
         <v>3</v>
       </c>
-      <c r="C36" s="130" t="s">
+      <c r="C36" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E36" s="18">
@@ -11570,7 +11576,7 @@
       <c r="B37" s="39">
         <v>3</v>
       </c>
-      <c r="C37" s="130" t="s">
+      <c r="C37" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E37" s="111">
@@ -11593,7 +11599,7 @@
       <c r="B38" s="39">
         <v>3</v>
       </c>
-      <c r="C38" s="130" t="s">
+      <c r="C38" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E38" s="18">
@@ -11616,7 +11622,7 @@
       <c r="B39" s="39">
         <v>5</v>
       </c>
-      <c r="C39" s="130" t="s">
+      <c r="C39" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E39" s="111">
@@ -11639,7 +11645,7 @@
       <c r="B40" s="39">
         <v>5</v>
       </c>
-      <c r="C40" s="130" t="s">
+      <c r="C40" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E40" s="18">
@@ -11662,7 +11668,7 @@
       <c r="B41" s="39">
         <v>3</v>
       </c>
-      <c r="C41" s="130" t="s">
+      <c r="C41" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E41" s="18">
@@ -11685,7 +11691,7 @@
       <c r="B42" s="39">
         <v>3</v>
       </c>
-      <c r="C42" s="130" t="s">
+      <c r="C42" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E42" s="18">
@@ -11708,7 +11714,7 @@
       <c r="B43" s="39">
         <v>2</v>
       </c>
-      <c r="C43" s="130" t="s">
+      <c r="C43" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E43" s="18">
@@ -11731,7 +11737,7 @@
       <c r="B44" s="39">
         <v>2</v>
       </c>
-      <c r="C44" s="130" t="s">
+      <c r="C44" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E44" s="18">
@@ -11754,7 +11760,7 @@
       <c r="B45" s="39">
         <v>2</v>
       </c>
-      <c r="C45" s="130" t="s">
+      <c r="C45" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E45" s="18">
@@ -11777,7 +11783,7 @@
       <c r="B46" s="39">
         <v>2</v>
       </c>
-      <c r="C46" s="130" t="s">
+      <c r="C46" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E46" s="18">
@@ -11800,7 +11806,7 @@
       <c r="B47" s="39">
         <v>1</v>
       </c>
-      <c r="C47" s="130" t="s">
+      <c r="C47" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E47" s="18">
@@ -11823,7 +11829,7 @@
       <c r="B48" s="19">
         <v>6</v>
       </c>
-      <c r="C48" s="130" t="s">
+      <c r="C48" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E48" s="111">
@@ -11846,7 +11852,7 @@
       <c r="B49" s="39">
         <v>5</v>
       </c>
-      <c r="C49" s="130" t="s">
+      <c r="C49" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E49" s="111">
@@ -11869,7 +11875,7 @@
       <c r="B50" s="39">
         <v>5</v>
       </c>
-      <c r="C50" s="130" t="s">
+      <c r="C50" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E50" s="18">
@@ -11892,7 +11898,7 @@
       <c r="B51" s="39">
         <v>5</v>
       </c>
-      <c r="C51" s="130" t="s">
+      <c r="C51" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E51" s="18">
@@ -11915,7 +11921,7 @@
       <c r="B52" s="39">
         <v>5</v>
       </c>
-      <c r="C52" s="130" t="s">
+      <c r="C52" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E52" s="18">
@@ -11936,12 +11942,12 @@
         <v>267</v>
       </c>
       <c r="B53" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C53" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D53" s="52" t="s">
+      <c r="D53" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E53" s="111">
@@ -11964,7 +11970,7 @@
       <c r="B54" s="39">
         <v>4</v>
       </c>
-      <c r="C54" s="130" t="s">
+      <c r="C54" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E54" s="111">
@@ -11987,7 +11993,7 @@
       <c r="B55" s="19">
         <v>6</v>
       </c>
-      <c r="C55" s="130" t="s">
+      <c r="C55" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E55" s="111">
@@ -12010,7 +12016,7 @@
       <c r="B56" s="39">
         <v>3</v>
       </c>
-      <c r="C56" s="130" t="s">
+      <c r="C56" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E56" s="18">
@@ -12033,7 +12039,7 @@
       <c r="B57" s="39">
         <v>2</v>
       </c>
-      <c r="C57" s="130" t="s">
+      <c r="C57" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E57" s="18">
@@ -12056,7 +12062,7 @@
       <c r="B58" s="39">
         <v>2</v>
       </c>
-      <c r="C58" s="130" t="s">
+      <c r="C58" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E58" s="18">
@@ -12079,7 +12085,7 @@
       <c r="B59" s="39">
         <v>2</v>
       </c>
-      <c r="C59" s="130" t="s">
+      <c r="C59" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E59" s="18">
@@ -12102,7 +12108,7 @@
       <c r="B60" s="19">
         <v>6</v>
       </c>
-      <c r="C60" s="130" t="s">
+      <c r="C60" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E60" s="111">
@@ -12125,7 +12131,7 @@
       <c r="B61" s="19">
         <v>6</v>
       </c>
-      <c r="C61" s="130" t="s">
+      <c r="C61" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E61" s="111">
@@ -12148,7 +12154,7 @@
       <c r="B62" s="19">
         <v>6</v>
       </c>
-      <c r="C62" s="130" t="s">
+      <c r="C62" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E62" s="18">
@@ -12171,7 +12177,7 @@
       <c r="B63" s="19">
         <v>6</v>
       </c>
-      <c r="C63" s="130" t="s">
+      <c r="C63" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E63" s="18">
@@ -12197,7 +12203,7 @@
       <c r="C64" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D64" s="52" t="s">
+      <c r="D64" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E64" s="111">
@@ -12220,7 +12226,7 @@
       <c r="B65" s="19">
         <v>6</v>
       </c>
-      <c r="C65" s="130" t="s">
+      <c r="C65" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E65" s="111">
@@ -12266,7 +12272,7 @@
       <c r="B67" s="39">
         <v>5</v>
       </c>
-      <c r="C67" s="130" t="s">
+      <c r="C67" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E67" s="111">
@@ -12289,7 +12295,7 @@
       <c r="B68" s="39">
         <v>4</v>
       </c>
-      <c r="C68" s="130" t="s">
+      <c r="C68" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E68" s="18">
@@ -12312,7 +12318,7 @@
       <c r="B69" s="39">
         <v>4</v>
       </c>
-      <c r="C69" s="130" t="s">
+      <c r="C69" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E69" s="18">
@@ -12358,7 +12364,7 @@
       <c r="B71" s="39">
         <v>2</v>
       </c>
-      <c r="C71" s="130" t="s">
+      <c r="C71" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E71" s="111">
@@ -12381,7 +12387,7 @@
       <c r="B72" s="39">
         <v>1</v>
       </c>
-      <c r="C72" s="130" t="s">
+      <c r="C72" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E72" s="18">
@@ -12404,7 +12410,7 @@
       <c r="B73" s="39">
         <v>3</v>
       </c>
-      <c r="C73" s="130" t="s">
+      <c r="C73" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E73" s="111">
@@ -12427,7 +12433,7 @@
       <c r="B74" s="39">
         <v>2</v>
       </c>
-      <c r="C74" s="130" t="s">
+      <c r="C74" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E74" s="18">
@@ -12450,7 +12456,7 @@
       <c r="B75" s="19">
         <v>6</v>
       </c>
-      <c r="C75" s="130" t="s">
+      <c r="C75" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E75" s="111">
@@ -12473,7 +12479,7 @@
       <c r="B76" s="39">
         <v>4</v>
       </c>
-      <c r="C76" s="130" t="s">
+      <c r="C76" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E76" s="18">
@@ -12496,7 +12502,7 @@
       <c r="B77" s="39">
         <v>4</v>
       </c>
-      <c r="C77" s="130" t="s">
+      <c r="C77" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E77" s="18">
@@ -12519,7 +12525,7 @@
       <c r="B78" s="19">
         <v>6</v>
       </c>
-      <c r="C78" s="130" t="s">
+      <c r="C78" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E78" s="111">
@@ -12542,7 +12548,7 @@
       <c r="B79" s="19">
         <v>6</v>
       </c>
-      <c r="C79" s="130" t="s">
+      <c r="C79" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E79" s="111">
@@ -12565,7 +12571,7 @@
       <c r="B80" s="19">
         <v>6</v>
       </c>
-      <c r="C80" s="130" t="s">
+      <c r="C80" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E80" s="18">
@@ -12614,7 +12620,7 @@
       <c r="C82" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D82" s="52" t="s">
+      <c r="D82" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E82" s="111">
@@ -12640,7 +12646,7 @@
       <c r="C83" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D83" s="52" t="s">
+      <c r="D83" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E83" s="18">
@@ -12666,7 +12672,7 @@
       <c r="C84" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D84" s="52" t="s">
+      <c r="D84" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E84" s="18">
@@ -12692,7 +12698,7 @@
       <c r="C85" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D85" s="52" t="s">
+      <c r="D85" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E85" s="18">
@@ -13060,7 +13066,7 @@
       <c r="B101" s="19">
         <v>6</v>
       </c>
-      <c r="C101" s="130" t="s">
+      <c r="C101" s="129" t="s">
         <v>276</v>
       </c>
       <c r="E101" s="18">
@@ -13086,7 +13092,7 @@
       <c r="C102" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D102" s="52" t="s">
+      <c r="D102" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E102" s="18">
@@ -13434,7 +13440,7 @@
       <c r="C117" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D117" s="52" t="s">
+      <c r="D117" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E117" s="18">
@@ -13460,7 +13466,7 @@
       <c r="C118" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D118" s="52" t="s">
+      <c r="D118" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E118" s="18">
@@ -13486,7 +13492,7 @@
       <c r="C119" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D119" s="52" t="s">
+      <c r="D119" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E119" s="18">
@@ -13512,7 +13518,7 @@
       <c r="C120" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D120" s="52" t="s">
+      <c r="D120" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E120" s="18">
@@ -13538,7 +13544,7 @@
       <c r="C121" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D121" s="52" t="s">
+      <c r="D121" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E121" s="18">
@@ -13564,7 +13570,7 @@
       <c r="C122" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D122" s="52" t="s">
+      <c r="D122" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E122" s="111">
@@ -13590,7 +13596,7 @@
       <c r="C123" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D123" s="52" t="s">
+      <c r="D123" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E123" s="18">
@@ -13800,7 +13806,7 @@
       <c r="C132" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D132" s="52" t="s">
+      <c r="D132" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E132" s="111">
@@ -13826,7 +13832,7 @@
       <c r="C133" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D133" s="52" t="s">
+      <c r="D133" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E133" s="18">
@@ -13941,7 +13947,7 @@
       <c r="B138" s="19">
         <v>6</v>
       </c>
-      <c r="C138" s="130" t="s">
+      <c r="C138" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E138" s="111">
@@ -14010,7 +14016,7 @@
       <c r="B141" s="19">
         <v>6</v>
       </c>
-      <c r="C141" s="130" t="s">
+      <c r="C141" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E141" s="111">
@@ -14033,7 +14039,7 @@
       <c r="B142" s="19">
         <v>6</v>
       </c>
-      <c r="C142" s="130" t="s">
+      <c r="C142" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E142" s="46">
@@ -14125,7 +14131,7 @@
       <c r="B146" s="39">
         <v>3</v>
       </c>
-      <c r="C146" s="130" t="s">
+      <c r="C146" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E146" s="111">
@@ -14151,7 +14157,7 @@
       <c r="C147" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D147" s="52" t="s">
+      <c r="D147" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E147" s="111">
@@ -14177,7 +14183,7 @@
       <c r="C148" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D148" s="52" t="s">
+      <c r="D148" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E148" s="111">
@@ -14272,7 +14278,7 @@
       <c r="C152" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D152" s="52" t="s">
+      <c r="D152" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E152" s="18">
@@ -14298,7 +14304,7 @@
       <c r="C153" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D153" s="52" t="s">
+      <c r="D153" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E153" s="111">
@@ -14324,7 +14330,7 @@
       <c r="C154" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D154" s="52" t="s">
+      <c r="D154" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E154" s="111">
@@ -14350,7 +14356,7 @@
       <c r="C155" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D155" s="52" t="s">
+      <c r="D155" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E155" s="18">
@@ -14376,7 +14382,7 @@
       <c r="C156" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D156" s="52" t="s">
+      <c r="D156" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E156" s="111">
@@ -14402,7 +14408,7 @@
       <c r="C157" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D157" s="52" t="s">
+      <c r="D157" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E157" s="111">
@@ -14428,7 +14434,7 @@
       <c r="C158" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D158" s="52" t="s">
+      <c r="D158" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E158" s="111">
@@ -14454,7 +14460,7 @@
       <c r="C159" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D159" s="52" t="s">
+      <c r="D159" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E159" s="111">
@@ -14480,7 +14486,7 @@
       <c r="C160" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D160" s="52" t="s">
+      <c r="D160" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E160" s="18">
@@ -14506,7 +14512,7 @@
       <c r="C161" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D161" s="52" t="s">
+      <c r="D161" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E161" s="18">
@@ -14532,7 +14538,7 @@
       <c r="C162" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D162" s="52" t="s">
+      <c r="D162" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E162" s="111">
@@ -14581,7 +14587,7 @@
       <c r="C164" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D164" s="52" t="s">
+      <c r="D164" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E164" s="111">
@@ -14607,7 +14613,7 @@
       <c r="C165" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D165" s="52" t="s">
+      <c r="D165" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E165" s="111">
@@ -14630,7 +14636,7 @@
       <c r="B166" s="19">
         <v>6</v>
       </c>
-      <c r="C166" s="130" t="s">
+      <c r="C166" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E166" s="111">
@@ -14674,12 +14680,12 @@
         <v>267</v>
       </c>
       <c r="B168" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C168" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D168" s="52" t="s">
+      <c r="D168" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E168" s="111">
@@ -14705,7 +14711,7 @@
       <c r="C169" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D169" s="52" t="s">
+      <c r="D169" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E169" s="18">
@@ -14772,12 +14778,12 @@
         <v>267</v>
       </c>
       <c r="B172" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C172" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D172" s="52" t="s">
+      <c r="D172" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E172" s="18">
@@ -14803,7 +14809,7 @@
       <c r="C173" s="113" t="s">
         <v>273</v>
       </c>
-      <c r="D173" s="52" t="s">
+      <c r="D173" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E173" s="114">
@@ -15008,12 +15014,12 @@
         <v>267</v>
       </c>
       <c r="B182" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C182" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D182" s="52" t="s">
+      <c r="D182" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E182" s="18">
@@ -15039,7 +15045,7 @@
       <c r="C183" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D183" s="52" t="s">
+      <c r="D183" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E183" s="18">
@@ -15060,12 +15066,12 @@
         <v>267</v>
       </c>
       <c r="B184" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C184" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D184" s="52" t="s">
+      <c r="D184" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E184" s="18">
@@ -15091,7 +15097,7 @@
       <c r="C185" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D185" s="52" t="s">
+      <c r="D185" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E185" s="111">
@@ -15135,12 +15141,12 @@
         <v>267</v>
       </c>
       <c r="B187" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C187" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D187" s="52" t="s">
+      <c r="D187" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E187" s="18">
@@ -15212,7 +15218,7 @@
       <c r="C190" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D190" s="52" t="s">
+      <c r="D190" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E190" s="111">
@@ -15284,7 +15290,7 @@
       <c r="C193" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D193" s="52" t="s">
+      <c r="D193" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E193" s="18">
@@ -15310,7 +15316,7 @@
       <c r="C194" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D194" s="52" t="s">
+      <c r="D194" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E194" s="111">
@@ -15474,7 +15480,7 @@
       <c r="C201" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D201" s="52" t="s">
+      <c r="D201" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E201" s="111">
@@ -15541,12 +15547,12 @@
         <v>267</v>
       </c>
       <c r="B204" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C204" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D204" s="52" t="s">
+      <c r="D204" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E204" s="111">
@@ -15641,7 +15647,7 @@
       <c r="C208" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D208" s="52" t="s">
+      <c r="D208" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E208" s="111">
@@ -15667,7 +15673,7 @@
       <c r="C209" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D209" s="52" t="s">
+      <c r="D209" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E209" s="111">
@@ -15693,7 +15699,7 @@
       <c r="C210" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D210" s="52" t="s">
+      <c r="D210" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E210" s="18">
@@ -15719,7 +15725,7 @@
       <c r="C211" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D211" s="52" t="s">
+      <c r="D211" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E211" s="18">
@@ -15740,12 +15746,12 @@
         <v>267</v>
       </c>
       <c r="B212" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C212" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D212" s="52" t="s">
+      <c r="D212" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E212" s="18">
@@ -15771,7 +15777,7 @@
       <c r="C213" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D213" s="52" t="s">
+      <c r="D213" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E213" s="18">
@@ -15797,7 +15803,7 @@
       <c r="C214" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D214" s="52" t="s">
+      <c r="D214" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E214" s="18">
@@ -15818,12 +15824,12 @@
         <v>267</v>
       </c>
       <c r="B215" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C215" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D215" s="52" t="s">
+      <c r="D215" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E215" s="18">
@@ -15849,7 +15855,7 @@
       <c r="C216" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D216" s="52" t="s">
+      <c r="D216" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E216" s="18">
@@ -15875,7 +15881,7 @@
       <c r="C217" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D217" s="52" t="s">
+      <c r="D217" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E217" s="18">
@@ -15901,7 +15907,7 @@
       <c r="C218" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D218" s="52" t="s">
+      <c r="D218" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E218" s="18">
@@ -15927,7 +15933,7 @@
       <c r="C219" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D219" s="52" t="s">
+      <c r="D219" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E219" s="18">
@@ -15953,7 +15959,7 @@
       <c r="C220" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D220" s="52" t="s">
+      <c r="D220" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E220" s="18">
@@ -15979,7 +15985,7 @@
       <c r="C221" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D221" s="52" t="s">
+      <c r="D221" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E221" s="18">
@@ -16000,12 +16006,12 @@
         <v>267</v>
       </c>
       <c r="B222" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C222" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D222" s="52" t="s">
+      <c r="D222" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E222" s="18">
@@ -16026,12 +16032,12 @@
         <v>267</v>
       </c>
       <c r="B223" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C223" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D223" s="52" t="s">
+      <c r="D223" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E223" s="18">
@@ -16052,12 +16058,12 @@
         <v>267</v>
       </c>
       <c r="B224" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C224" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D224" s="52" t="s">
+      <c r="D224" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E224" s="18">
@@ -16106,7 +16112,7 @@
       <c r="C226" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D226" s="52" t="s">
+      <c r="D226" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E226" s="18">
@@ -16132,7 +16138,7 @@
       <c r="C227" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D227" s="52" t="s">
+      <c r="D227" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E227" s="111">
@@ -16153,12 +16159,12 @@
         <v>267</v>
       </c>
       <c r="B228" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C228" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D228" s="52" t="s">
+      <c r="D228" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E228" s="111">
@@ -16179,12 +16185,12 @@
         <v>267</v>
       </c>
       <c r="B229" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C229" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D229" s="52" t="s">
+      <c r="D229" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E229" s="18">
@@ -16210,7 +16216,7 @@
       <c r="C230" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D230" s="52" t="s">
+      <c r="D230" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E230" s="111">
@@ -16236,7 +16242,7 @@
       <c r="C231" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D231" s="52" t="s">
+      <c r="D231" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E231" s="18">
@@ -16262,7 +16268,7 @@
       <c r="C232" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D232" s="52" t="s">
+      <c r="D232" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E232" s="18">
@@ -16283,12 +16289,12 @@
         <v>267</v>
       </c>
       <c r="B233" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C233" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D233" s="52" t="s">
+      <c r="D233" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E233" s="18">
@@ -16314,7 +16320,7 @@
       <c r="C234" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D234" s="52" t="s">
+      <c r="D234" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E234" s="18">
@@ -16340,7 +16346,7 @@
       <c r="C235" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D235" s="52" t="s">
+      <c r="D235" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E235" s="18">
@@ -16366,7 +16372,7 @@
       <c r="C236" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D236" s="52" t="s">
+      <c r="D236" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E236" s="111">
@@ -16412,7 +16418,7 @@
       <c r="B238" s="19">
         <v>6</v>
       </c>
-      <c r="C238" s="130" t="s">
+      <c r="C238" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E238" s="18">
@@ -16438,7 +16444,7 @@
       <c r="C239" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D239" s="52" t="s">
+      <c r="D239" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E239" s="111">
@@ -16482,12 +16488,12 @@
         <v>267</v>
       </c>
       <c r="B241" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C241" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D241" s="52" t="s">
+      <c r="D241" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E241" s="18">
@@ -16508,12 +16514,12 @@
         <v>267</v>
       </c>
       <c r="B242" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C242" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D242" s="52" t="s">
+      <c r="D242" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E242" s="18">
@@ -16534,12 +16540,12 @@
         <v>267</v>
       </c>
       <c r="B243" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C243" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D243" s="52" t="s">
+      <c r="D243" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E243" s="18">
@@ -16565,7 +16571,7 @@
       <c r="C244" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D244" s="52" t="s">
+      <c r="D244" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E244" s="18">
@@ -16591,7 +16597,7 @@
       <c r="C245" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D245" s="52" t="s">
+      <c r="D245" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E245" s="18">
@@ -16617,7 +16623,7 @@
       <c r="C246" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D246" s="52" t="s">
+      <c r="D246" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E246" s="18">
@@ -16643,7 +16649,7 @@
       <c r="C247" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D247" s="52" t="s">
+      <c r="D247" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E247" s="111">
@@ -16784,7 +16790,7 @@
       <c r="C253" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D253" s="52" t="s">
+      <c r="D253" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E253" s="18">
@@ -16810,7 +16816,7 @@
       <c r="C254" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D254" s="52" t="s">
+      <c r="D254" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E254" s="18">
@@ -16836,7 +16842,7 @@
       <c r="C255" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D255" s="52" t="s">
+      <c r="D255" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E255" s="18">
@@ -16862,7 +16868,7 @@
       <c r="C256" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D256" s="127" t="s">
+      <c r="D256" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E256" s="18">
@@ -16888,7 +16894,7 @@
       <c r="C257" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D257" s="127" t="s">
+      <c r="D257" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E257" s="18">
@@ -16914,7 +16920,7 @@
       <c r="C258" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D258" s="52" t="s">
+      <c r="D258" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E258" s="18">
@@ -16940,7 +16946,7 @@
       <c r="C259" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D259" s="52" t="s">
+      <c r="D259" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E259" s="18">
@@ -16966,7 +16972,7 @@
       <c r="C260" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D260" s="52" t="s">
+      <c r="D260" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E260" s="18">
@@ -16987,12 +16993,12 @@
         <v>267</v>
       </c>
       <c r="B261" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C261" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D261" s="52" t="s">
+      <c r="D261" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E261" s="18">
@@ -17013,12 +17019,12 @@
         <v>267</v>
       </c>
       <c r="B262" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C262" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D262" s="52" t="s">
+      <c r="D262" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E262" s="18">
@@ -17039,12 +17045,12 @@
         <v>267</v>
       </c>
       <c r="B263" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C263" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D263" s="52" t="s">
+      <c r="D263" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E263" s="18">
@@ -17065,12 +17071,12 @@
         <v>267</v>
       </c>
       <c r="B264" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C264" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D264" s="52" t="s">
+      <c r="D264" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E264" s="111">
@@ -17096,7 +17102,7 @@
       <c r="C265" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D265" s="52" t="s">
+      <c r="D265" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E265" s="18">
@@ -17122,7 +17128,7 @@
       <c r="C266" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D266" s="52" t="s">
+      <c r="D266" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E266" s="18">
@@ -17189,12 +17195,12 @@
         <v>267</v>
       </c>
       <c r="B269" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C269" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D269" s="52" t="s">
+      <c r="D269" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E269" s="111">
@@ -17215,12 +17221,12 @@
         <v>267</v>
       </c>
       <c r="B270" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C270" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D270" s="52" t="s">
+      <c r="D270" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E270" s="111">
@@ -17269,7 +17275,7 @@
       <c r="C272" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D272" s="52" t="s">
+      <c r="D272" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E272" s="111">
@@ -17295,7 +17301,7 @@
       <c r="C273" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D273" s="52" t="s">
+      <c r="D273" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E273" s="18">
@@ -17321,7 +17327,7 @@
       <c r="C274" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D274" s="52" t="s">
+      <c r="D274" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E274" s="18">
@@ -17347,7 +17353,7 @@
       <c r="C275" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D275" s="52" t="s">
+      <c r="D275" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E275" s="18">
@@ -17511,7 +17517,7 @@
       <c r="C282" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D282" s="52" t="s">
+      <c r="D282" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E282" s="18">
@@ -17532,12 +17538,12 @@
         <v>267</v>
       </c>
       <c r="B283" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C283" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D283" s="52" t="s">
+      <c r="D283" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E283" s="18">
@@ -17586,7 +17592,7 @@
       <c r="C285" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D285" s="52" t="s">
+      <c r="D285" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E285" s="111">
@@ -17612,7 +17618,7 @@
       <c r="C286" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D286" s="52" t="s">
+      <c r="D286" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E286" s="111">
@@ -17730,7 +17736,7 @@
       <c r="C291" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D291" s="52" t="s">
+      <c r="D291" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E291" s="111">
@@ -17779,7 +17785,7 @@
       <c r="C293" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D293" s="52" t="s">
+      <c r="D293" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E293" s="111">
@@ -17894,7 +17900,7 @@
       <c r="B298" s="19">
         <v>6</v>
       </c>
-      <c r="C298" s="130" t="s">
+      <c r="C298" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E298" s="18">
@@ -17915,12 +17921,12 @@
         <v>267</v>
       </c>
       <c r="B299" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C299" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D299" s="52" t="s">
+      <c r="D299" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E299" s="18">
@@ -17946,7 +17952,7 @@
       <c r="C300" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D300" s="52" t="s">
+      <c r="D300" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E300" s="18">
@@ -17967,12 +17973,12 @@
         <v>267</v>
       </c>
       <c r="B301" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C301" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D301" s="52" t="s">
+      <c r="D301" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E301" s="18">
@@ -17998,7 +18004,7 @@
       <c r="C302" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D302" s="52" t="s">
+      <c r="D302" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E302" s="18">
@@ -18088,12 +18094,12 @@
         <v>267</v>
       </c>
       <c r="B306" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C306" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D306" s="52" t="s">
+      <c r="D306" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E306" s="115">
@@ -18119,7 +18125,7 @@
       <c r="C307" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D307" s="52" t="s">
+      <c r="D307" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E307" s="18">
@@ -18145,7 +18151,7 @@
       <c r="C308" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D308" s="52" t="s">
+      <c r="D308" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E308" s="18">
@@ -18171,7 +18177,7 @@
       <c r="C309" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D309" s="52" t="s">
+      <c r="D309" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E309" s="18">
@@ -18197,7 +18203,7 @@
       <c r="C310" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D310" s="52" t="s">
+      <c r="D310" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E310" s="18">
@@ -18218,12 +18224,12 @@
         <v>267</v>
       </c>
       <c r="B311" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C311" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D311" s="52" t="s">
+      <c r="D311" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E311" s="18">
@@ -18341,7 +18347,7 @@
       <c r="C316" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D316" s="52" t="s">
+      <c r="D316" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E316" s="111">
@@ -18367,7 +18373,7 @@
       <c r="C317" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D317" s="52" t="s">
+      <c r="D317" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E317" s="111">
@@ -18393,7 +18399,7 @@
       <c r="C318" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D318" s="52" t="s">
+      <c r="D318" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E318" s="111">
@@ -18442,7 +18448,7 @@
       <c r="C320" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D320" s="52" t="s">
+      <c r="D320" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E320" s="111">
@@ -18537,7 +18543,7 @@
       <c r="C324" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D324" s="52" t="s">
+      <c r="D324" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E324" s="111">
@@ -18560,7 +18566,7 @@
       <c r="B325" s="39">
         <v>1</v>
       </c>
-      <c r="C325" s="130" t="s">
+      <c r="C325" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E325" s="111">
@@ -18583,7 +18589,7 @@
       <c r="B326" s="39">
         <v>1</v>
       </c>
-      <c r="C326" s="130" t="s">
+      <c r="C326" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E326" s="18">
@@ -18606,7 +18612,7 @@
       <c r="B327" s="39">
         <v>1</v>
       </c>
-      <c r="C327" s="130" t="s">
+      <c r="C327" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E327" s="18">
@@ -18629,7 +18635,7 @@
       <c r="B328" s="19">
         <v>6</v>
       </c>
-      <c r="C328" s="130" t="s">
+      <c r="C328" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E328" s="111">
@@ -18652,7 +18658,7 @@
       <c r="B329" s="39">
         <v>2</v>
       </c>
-      <c r="C329" s="130" t="s">
+      <c r="C329" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E329" s="111">
@@ -18675,7 +18681,7 @@
       <c r="B330" s="19">
         <v>6</v>
       </c>
-      <c r="C330" s="130" t="s">
+      <c r="C330" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E330" s="111">
@@ -18698,7 +18704,7 @@
       <c r="B331" s="19">
         <v>6</v>
       </c>
-      <c r="C331" s="130" t="s">
+      <c r="C331" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E331" s="18">
@@ -18721,7 +18727,7 @@
       <c r="B332" s="39">
         <v>5</v>
       </c>
-      <c r="C332" s="130" t="s">
+      <c r="C332" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E332" s="18">
@@ -18744,7 +18750,7 @@
       <c r="B333" s="39">
         <v>5</v>
       </c>
-      <c r="C333" s="130" t="s">
+      <c r="C333" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E333" s="111">
@@ -18793,7 +18799,7 @@
       <c r="C335" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D335" s="52" t="s">
+      <c r="D335" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E335" s="111">
@@ -18819,7 +18825,7 @@
       <c r="C336" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D336" s="52" t="s">
+      <c r="D336" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E336" s="111">
@@ -18842,7 +18848,7 @@
       <c r="B337" s="39">
         <v>1</v>
       </c>
-      <c r="C337" s="130" t="s">
+      <c r="C337" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E337" s="111">
@@ -18865,7 +18871,7 @@
       <c r="B338" s="39">
         <v>1</v>
       </c>
-      <c r="C338" s="130" t="s">
+      <c r="C338" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E338" s="18">
@@ -18937,7 +18943,7 @@
       <c r="C341" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D341" s="52" t="s">
+      <c r="D341" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E341" s="111">
@@ -18960,7 +18966,7 @@
       <c r="B342" s="19">
         <v>6</v>
       </c>
-      <c r="C342" s="130" t="s">
+      <c r="C342" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E342" s="111">
@@ -19006,7 +19012,7 @@
       <c r="B344" s="19">
         <v>6</v>
       </c>
-      <c r="C344" s="130" t="s">
+      <c r="C344" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E344" s="111">
@@ -19029,7 +19035,7 @@
       <c r="B345" s="19">
         <v>6</v>
       </c>
-      <c r="C345" s="130" t="s">
+      <c r="C345" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E345" s="111">
@@ -19052,7 +19058,7 @@
       <c r="B346" s="19">
         <v>6</v>
       </c>
-      <c r="C346" s="130" t="s">
+      <c r="C346" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E346" s="111">
@@ -19121,7 +19127,7 @@
       <c r="B349" s="19">
         <v>6</v>
       </c>
-      <c r="C349" s="130" t="s">
+      <c r="C349" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E349" s="111">
@@ -19144,7 +19150,7 @@
       <c r="B350" s="19">
         <v>6</v>
       </c>
-      <c r="C350" s="130" t="s">
+      <c r="C350" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E350" s="111">
@@ -19170,7 +19176,7 @@
       <c r="C351" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D351" s="52" t="s">
+      <c r="D351" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E351" s="111">
@@ -19239,7 +19245,7 @@
       <c r="B354" s="19">
         <v>6</v>
       </c>
-      <c r="C354" s="130" t="s">
+      <c r="C354" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E354" s="18">
@@ -19265,7 +19271,7 @@
       <c r="C355" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D355" s="52" t="s">
+      <c r="D355" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E355" s="111">
@@ -19521,7 +19527,7 @@
       <c r="C366" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D366" s="52" t="s">
+      <c r="D366" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E366" s="111">
@@ -19547,7 +19553,7 @@
       <c r="C367" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D367" s="52" t="s">
+      <c r="D367" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E367" s="111">
@@ -19573,7 +19579,7 @@
       <c r="C368" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D368" s="52" t="s">
+      <c r="D368" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E368" s="18">
@@ -19599,7 +19605,7 @@
       <c r="C369" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D369" s="52" t="s">
+      <c r="D369" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E369" s="18">
@@ -19625,7 +19631,7 @@
       <c r="C370" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D370" s="52" t="s">
+      <c r="D370" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E370" s="18">
@@ -19646,12 +19652,12 @@
         <v>267</v>
       </c>
       <c r="B371" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C371" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D371" s="52" t="s">
+      <c r="D371" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E371" s="18">
@@ -19674,7 +19680,7 @@
       <c r="B372" s="19">
         <v>6</v>
       </c>
-      <c r="C372" s="130" t="s">
+      <c r="C372" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E372" s="18">
@@ -19769,7 +19775,7 @@
       <c r="C376" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D376" s="52" t="s">
+      <c r="D376" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E376" s="111">
@@ -19790,12 +19796,12 @@
         <v>267</v>
       </c>
       <c r="B377" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C377" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D377" s="52" t="s">
+      <c r="D377" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E377" s="18">
@@ -19821,7 +19827,7 @@
       <c r="C378" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D378" s="52" t="s">
+      <c r="D378" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E378" s="18">
@@ -19847,7 +19853,7 @@
       <c r="C379" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D379" s="52" t="s">
+      <c r="D379" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E379" s="18">
@@ -19873,7 +19879,7 @@
       <c r="C380" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D380" s="52" t="s">
+      <c r="D380" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E380" s="18">
@@ -19894,12 +19900,12 @@
         <v>267</v>
       </c>
       <c r="B381" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C381" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D381" s="52" t="s">
+      <c r="D381" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E381" s="18">
@@ -19920,12 +19926,12 @@
         <v>267</v>
       </c>
       <c r="B382" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C382" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D382" s="52" t="s">
+      <c r="D382" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E382" s="111">
@@ -19946,12 +19952,12 @@
         <v>267</v>
       </c>
       <c r="B383" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C383" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D383" s="52" t="s">
+      <c r="D383" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E383" s="18">
@@ -19972,12 +19978,12 @@
         <v>267</v>
       </c>
       <c r="B384" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C384" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D384" s="52" t="s">
+      <c r="D384" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E384" s="18">
@@ -19998,12 +20004,12 @@
         <v>267</v>
       </c>
       <c r="B385" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C385" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D385" s="52" t="s">
+      <c r="D385" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E385" s="111">
@@ -20024,12 +20030,12 @@
         <v>267</v>
       </c>
       <c r="B386" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C386" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D386" s="52" t="s">
+      <c r="D386" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E386" s="18">
@@ -20239,7 +20245,7 @@
       <c r="C395" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D395" s="52" t="s">
+      <c r="D395" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E395" s="18">
@@ -20265,7 +20271,7 @@
       <c r="C396" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D396" s="52" t="s">
+      <c r="D396" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E396" s="18">
@@ -20291,7 +20297,7 @@
       <c r="C397" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D397" s="52" t="s">
+      <c r="D397" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E397" s="111">
@@ -20317,7 +20323,7 @@
       <c r="C398" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D398" s="52" t="s">
+      <c r="D398" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E398" s="18">
@@ -20343,7 +20349,7 @@
       <c r="C399" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D399" s="52" t="s">
+      <c r="D399" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E399" s="18">
@@ -20369,7 +20375,7 @@
       <c r="C400" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D400" s="52" t="s">
+      <c r="D400" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E400" s="18">
@@ -20395,7 +20401,7 @@
       <c r="C401" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D401" s="52" t="s">
+      <c r="D401" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E401" s="18">
@@ -20416,12 +20422,12 @@
         <v>267</v>
       </c>
       <c r="B402" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C402" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D402" s="52" t="s">
+      <c r="D402" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E402" s="18">
@@ -20442,12 +20448,12 @@
         <v>267</v>
       </c>
       <c r="B403" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C403" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D403" s="52" t="s">
+      <c r="D403" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E403" s="18">
@@ -20468,12 +20474,12 @@
         <v>267</v>
       </c>
       <c r="B404" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C404" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D404" s="52" t="s">
+      <c r="D404" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E404" s="18">
@@ -20494,12 +20500,12 @@
         <v>267</v>
       </c>
       <c r="B405" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C405" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D405" s="52" t="s">
+      <c r="D405" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E405" s="18">
@@ -20525,7 +20531,7 @@
       <c r="C406" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D406" s="52" t="s">
+      <c r="D406" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E406" s="18">
@@ -20551,7 +20557,7 @@
       <c r="C407" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D407" s="52" t="s">
+      <c r="D407" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E407" s="18">
@@ -20577,7 +20583,7 @@
       <c r="C408" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D408" s="52" t="s">
+      <c r="D408" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E408" s="18">
@@ -20603,7 +20609,7 @@
       <c r="C409" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D409" s="52" t="s">
+      <c r="D409" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E409" s="111">
@@ -20624,12 +20630,12 @@
         <v>267</v>
       </c>
       <c r="B410" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C410" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D410" s="52" t="s">
+      <c r="D410" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E410" s="18">
@@ -20655,7 +20661,7 @@
       <c r="C411" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D411" s="52" t="s">
+      <c r="D411" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E411" s="111">
@@ -20681,7 +20687,7 @@
       <c r="C412" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D412" s="52" t="s">
+      <c r="D412" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E412" s="18">
@@ -20707,7 +20713,7 @@
       <c r="C413" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D413" s="52" t="s">
+      <c r="D413" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E413" s="18">
@@ -20733,7 +20739,7 @@
       <c r="C414" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D414" s="52" t="s">
+      <c r="D414" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E414" s="18">
@@ -20759,7 +20765,7 @@
       <c r="C415" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D415" s="52" t="s">
+      <c r="D415" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E415" s="18">
@@ -20785,7 +20791,7 @@
       <c r="C416" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D416" s="52" t="s">
+      <c r="D416" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E416" s="18">
@@ -20811,7 +20817,7 @@
       <c r="C417" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D417" s="52" t="s">
+      <c r="D417" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E417" s="18">
@@ -20860,7 +20866,7 @@
       <c r="C419" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D419" s="52" t="s">
+      <c r="D419" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E419" s="111">
@@ -20886,7 +20892,7 @@
       <c r="C420" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D420" s="52" t="s">
+      <c r="D420" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E420" s="18">
@@ -20958,7 +20964,7 @@
       <c r="C423" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D423" s="52" t="s">
+      <c r="D423" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E423" s="18">
@@ -20984,7 +20990,7 @@
       <c r="C424" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D424" s="52" t="s">
+      <c r="D424" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E424" s="18">
@@ -21010,7 +21016,7 @@
       <c r="C425" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D425" s="52" t="s">
+      <c r="D425" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E425" s="111">
@@ -21036,7 +21042,7 @@
       <c r="C426" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D426" s="52" t="s">
+      <c r="D426" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E426" s="111">
@@ -21062,7 +21068,7 @@
       <c r="C427" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D427" s="52" t="s">
+      <c r="D427" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E427" s="111">
@@ -21088,7 +21094,7 @@
       <c r="C428" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D428" s="52" t="s">
+      <c r="D428" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E428" s="18">
@@ -21114,7 +21120,7 @@
       <c r="C429" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D429" s="52" t="s">
+      <c r="D429" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E429" s="111">
@@ -21140,7 +21146,7 @@
       <c r="C430" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D430" s="52" t="s">
+      <c r="D430" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E430" s="18">
@@ -21276,12 +21282,12 @@
         <v>267</v>
       </c>
       <c r="B436" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C436" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D436" s="52" t="s">
+      <c r="D436" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E436" s="111">
@@ -21330,7 +21336,7 @@
       <c r="C438" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D438" s="52" t="s">
+      <c r="D438" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E438" s="111">
@@ -21351,12 +21357,12 @@
         <v>267</v>
       </c>
       <c r="B439" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C439" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D439" s="52" t="s">
+      <c r="D439" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E439" s="18">
@@ -21382,7 +21388,7 @@
       <c r="C440" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D440" s="52" t="s">
+      <c r="D440" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E440" s="111">
@@ -21408,7 +21414,7 @@
       <c r="C441" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D441" s="52" t="s">
+      <c r="D441" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E441" s="18">
@@ -21457,7 +21463,7 @@
       <c r="C443" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D443" s="52" t="s">
+      <c r="D443" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E443" s="111">
@@ -21483,7 +21489,7 @@
       <c r="C444" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D444" s="52" t="s">
+      <c r="D444" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E444" s="111">
@@ -21532,7 +21538,7 @@
       <c r="C446" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D446" s="52" t="s">
+      <c r="D446" s="38" t="s">
         <v>1903</v>
       </c>
       <c r="E446" s="111">
@@ -21558,7 +21564,7 @@
       <c r="C447" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D447" s="52" t="s">
+      <c r="D447" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E447" s="111">
@@ -21579,12 +21585,12 @@
         <v>267</v>
       </c>
       <c r="B448" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C448" s="39" t="s">
         <v>277</v>
       </c>
-      <c r="D448" s="52" t="s">
+      <c r="D448" s="38" t="s">
         <v>1889</v>
       </c>
       <c r="E448" s="18">
@@ -21605,12 +21611,12 @@
         <v>267</v>
       </c>
       <c r="B449" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C449" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D449" s="52" t="s">
+      <c r="D449" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E449" s="18">
@@ -21702,7 +21708,7 @@
       <c r="B453" s="19">
         <v>6</v>
       </c>
-      <c r="C453" s="130" t="s">
+      <c r="C453" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E453" s="111">
@@ -21725,7 +21731,7 @@
       <c r="B454" s="19">
         <v>6</v>
       </c>
-      <c r="C454" s="130" t="s">
+      <c r="C454" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E454" s="18">
@@ -21748,7 +21754,7 @@
       <c r="B455" s="19">
         <v>6</v>
       </c>
-      <c r="C455" s="130" t="s">
+      <c r="C455" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E455" s="18">
@@ -21771,7 +21777,7 @@
       <c r="B456" s="19">
         <v>6</v>
       </c>
-      <c r="C456" s="130" t="s">
+      <c r="C456" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E456" s="18">
@@ -21794,7 +21800,7 @@
       <c r="B457" s="19">
         <v>6</v>
       </c>
-      <c r="C457" s="130" t="s">
+      <c r="C457" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E457" s="18">
@@ -21817,7 +21823,7 @@
       <c r="B458" s="19">
         <v>6</v>
       </c>
-      <c r="C458" s="130" t="s">
+      <c r="C458" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E458" s="18">
@@ -21840,7 +21846,7 @@
       <c r="B459" s="19">
         <v>6</v>
       </c>
-      <c r="C459" s="130" t="s">
+      <c r="C459" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E459" s="18">
@@ -21863,7 +21869,7 @@
       <c r="B460" s="39">
         <v>2</v>
       </c>
-      <c r="C460" s="130" t="s">
+      <c r="C460" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E460" s="18">
@@ -21886,7 +21892,7 @@
       <c r="B461" s="39">
         <v>5</v>
       </c>
-      <c r="C461" s="130" t="s">
+      <c r="C461" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E461" s="18">
@@ -21909,7 +21915,7 @@
       <c r="B462" s="19">
         <v>6</v>
       </c>
-      <c r="C462" s="130" t="s">
+      <c r="C462" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E462" s="18">
@@ -21932,7 +21938,7 @@
       <c r="B463" s="19">
         <v>6</v>
       </c>
-      <c r="C463" s="130" t="s">
+      <c r="C463" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E463" s="111">
@@ -21955,7 +21961,7 @@
       <c r="B464" s="19">
         <v>6</v>
       </c>
-      <c r="C464" s="130" t="s">
+      <c r="C464" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E464" s="111">
@@ -21981,7 +21987,7 @@
       <c r="C465" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D465" s="52" t="s">
+      <c r="D465" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E465" s="111">
@@ -22004,7 +22010,7 @@
       <c r="B466" s="19">
         <v>6</v>
       </c>
-      <c r="C466" s="130" t="s">
+      <c r="C466" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E466" s="18">
@@ -22027,7 +22033,7 @@
       <c r="B467" s="19">
         <v>6</v>
       </c>
-      <c r="C467" s="130" t="s">
+      <c r="C467" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E467" s="111">
@@ -22050,7 +22056,7 @@
       <c r="B468" s="39">
         <v>2</v>
       </c>
-      <c r="C468" s="130" t="s">
+      <c r="C468" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E468" s="18">
@@ -22073,7 +22079,7 @@
       <c r="B469" s="19">
         <v>6</v>
       </c>
-      <c r="C469" s="130" t="s">
+      <c r="C469" s="129" t="s">
         <v>276</v>
       </c>
       <c r="E469" s="111">
@@ -22096,7 +22102,7 @@
       <c r="B470" s="39">
         <v>2</v>
       </c>
-      <c r="C470" s="130" t="s">
+      <c r="C470" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E470" s="111">
@@ -22119,7 +22125,7 @@
       <c r="B471" s="19">
         <v>6</v>
       </c>
-      <c r="C471" s="130" t="s">
+      <c r="C471" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E471" s="111">
@@ -22142,7 +22148,7 @@
       <c r="B472" s="19">
         <v>6</v>
       </c>
-      <c r="C472" s="130" t="s">
+      <c r="C472" s="129" t="s">
         <v>276</v>
       </c>
       <c r="E472" s="18">
@@ -22165,7 +22171,7 @@
       <c r="B473" s="19">
         <v>6</v>
       </c>
-      <c r="C473" s="130" t="s">
+      <c r="C473" s="129" t="s">
         <v>276</v>
       </c>
       <c r="E473" s="18">
@@ -22188,7 +22194,7 @@
       <c r="B474" s="39">
         <v>5</v>
       </c>
-      <c r="C474" s="130" t="s">
+      <c r="C474" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E474" s="18">
@@ -22211,7 +22217,7 @@
       <c r="B475" s="39">
         <v>4</v>
       </c>
-      <c r="C475" s="130" t="s">
+      <c r="C475" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E475" s="18">
@@ -22234,7 +22240,7 @@
       <c r="B476" s="39">
         <v>3</v>
       </c>
-      <c r="C476" s="130" t="s">
+      <c r="C476" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E476" s="18">
@@ -22257,7 +22263,7 @@
       <c r="B477" s="39">
         <v>2</v>
       </c>
-      <c r="C477" s="130" t="s">
+      <c r="C477" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E477" s="18">
@@ -22280,7 +22286,7 @@
       <c r="B478" s="39">
         <v>2</v>
       </c>
-      <c r="C478" s="130" t="s">
+      <c r="C478" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E478" s="18">
@@ -22303,7 +22309,7 @@
       <c r="B479" s="39">
         <v>2</v>
       </c>
-      <c r="C479" s="130" t="s">
+      <c r="C479" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E479" s="18">
@@ -22326,7 +22332,7 @@
       <c r="B480" s="39">
         <v>2</v>
       </c>
-      <c r="C480" s="130" t="s">
+      <c r="C480" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E480" s="18">
@@ -22349,7 +22355,7 @@
       <c r="B481" s="39">
         <v>2</v>
       </c>
-      <c r="C481" s="130" t="s">
+      <c r="C481" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E481" s="18">
@@ -22372,7 +22378,7 @@
       <c r="B482" s="39">
         <v>2</v>
       </c>
-      <c r="C482" s="130" t="s">
+      <c r="C482" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E482" s="18">
@@ -22395,7 +22401,7 @@
       <c r="B483" s="39">
         <v>1</v>
       </c>
-      <c r="C483" s="130" t="s">
+      <c r="C483" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E483" s="18">
@@ -22418,7 +22424,7 @@
       <c r="B484" s="39">
         <v>1</v>
       </c>
-      <c r="C484" s="130" t="s">
+      <c r="C484" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E484" s="18">
@@ -22441,7 +22447,7 @@
       <c r="B485" s="39">
         <v>2</v>
       </c>
-      <c r="C485" s="130" t="s">
+      <c r="C485" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E485" s="111">
@@ -22464,7 +22470,7 @@
       <c r="B486" s="39">
         <v>4</v>
       </c>
-      <c r="C486" s="130" t="s">
+      <c r="C486" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E486" s="111">
@@ -22487,7 +22493,7 @@
       <c r="B487" s="39">
         <v>4</v>
       </c>
-      <c r="C487" s="130" t="s">
+      <c r="C487" s="129" t="s">
         <v>279</v>
       </c>
       <c r="E487" s="111">
@@ -22510,7 +22516,7 @@
       <c r="B488" s="19">
         <v>6</v>
       </c>
-      <c r="C488" s="130" t="s">
+      <c r="C488" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E488" s="111">
@@ -22533,7 +22539,7 @@
       <c r="B489" s="39">
         <v>2</v>
       </c>
-      <c r="C489" s="130" t="s">
+      <c r="C489" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E489" s="18">
@@ -22556,7 +22562,7 @@
       <c r="B490" s="39">
         <v>2</v>
       </c>
-      <c r="C490" s="130" t="s">
+      <c r="C490" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E490" s="18">
@@ -22579,7 +22585,7 @@
       <c r="B491" s="19">
         <v>6</v>
       </c>
-      <c r="C491" s="130" t="s">
+      <c r="C491" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E491" s="111">
@@ -22602,7 +22608,7 @@
       <c r="B492" s="19">
         <v>6</v>
       </c>
-      <c r="C492" s="130" t="s">
+      <c r="C492" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E492" s="18">
@@ -22625,7 +22631,7 @@
       <c r="B493" s="20">
         <v>6</v>
       </c>
-      <c r="C493" s="130" t="s">
+      <c r="C493" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E493" s="111">
@@ -22694,7 +22700,7 @@
       <c r="B496" s="19">
         <v>6</v>
       </c>
-      <c r="C496" s="130" t="s">
+      <c r="C496" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E496" s="111">
@@ -22717,7 +22723,7 @@
       <c r="B497" s="39">
         <v>3</v>
       </c>
-      <c r="C497" s="130" t="s">
+      <c r="C497" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E497" s="18">
@@ -22740,7 +22746,7 @@
       <c r="B498" s="19">
         <v>6</v>
       </c>
-      <c r="C498" s="130" t="s">
+      <c r="C498" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E498" s="18">
@@ -22763,7 +22769,7 @@
       <c r="B499" s="19">
         <v>6</v>
       </c>
-      <c r="C499" s="130" t="s">
+      <c r="C499" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E499" s="18">
@@ -22807,12 +22813,12 @@
         <v>267</v>
       </c>
       <c r="B501" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C501" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D501" s="52" t="s">
+      <c r="D501" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E501" s="111">
@@ -22881,7 +22887,7 @@
       <c r="B504" s="19">
         <v>6</v>
       </c>
-      <c r="C504" s="130" t="s">
+      <c r="C504" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E504" s="18">
@@ -22904,7 +22910,7 @@
       <c r="B505" s="39">
         <v>5</v>
       </c>
-      <c r="C505" s="130" t="s">
+      <c r="C505" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E505" s="18">
@@ -22927,7 +22933,7 @@
       <c r="B506" s="19">
         <v>6</v>
       </c>
-      <c r="C506" s="130" t="s">
+      <c r="C506" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E506" s="111">
@@ -22950,7 +22956,7 @@
       <c r="B507" s="19">
         <v>6</v>
       </c>
-      <c r="C507" s="130" t="s">
+      <c r="C507" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E507" s="18">
@@ -22973,7 +22979,7 @@
       <c r="B508" s="19">
         <v>6</v>
       </c>
-      <c r="C508" s="130" t="s">
+      <c r="C508" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E508" s="18">
@@ -22996,7 +23002,7 @@
       <c r="B509" s="19">
         <v>6</v>
       </c>
-      <c r="C509" s="130" t="s">
+      <c r="C509" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E509" s="18">
@@ -23019,7 +23025,7 @@
       <c r="B510" s="19">
         <v>6</v>
       </c>
-      <c r="C510" s="130" t="s">
+      <c r="C510" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E510" s="18">
@@ -23042,7 +23048,7 @@
       <c r="B511" s="19">
         <v>6</v>
       </c>
-      <c r="C511" s="130" t="s">
+      <c r="C511" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E511" s="18">
@@ -23065,7 +23071,7 @@
       <c r="B512" s="19">
         <v>6</v>
       </c>
-      <c r="C512" s="130" t="s">
+      <c r="C512" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E512" s="18">
@@ -23088,7 +23094,7 @@
       <c r="B513" s="19">
         <v>6</v>
       </c>
-      <c r="C513" s="130" t="s">
+      <c r="C513" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E513" s="18">
@@ -23111,7 +23117,7 @@
       <c r="B514" s="19">
         <v>6</v>
       </c>
-      <c r="C514" s="130" t="s">
+      <c r="C514" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E514" s="111">
@@ -23134,7 +23140,7 @@
       <c r="B515" s="19">
         <v>6</v>
       </c>
-      <c r="C515" s="130" t="s">
+      <c r="C515" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E515" s="18">
@@ -23157,7 +23163,7 @@
       <c r="B516" s="19">
         <v>6</v>
       </c>
-      <c r="C516" s="130" t="s">
+      <c r="C516" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E516" s="18">
@@ -23180,7 +23186,7 @@
       <c r="B517" s="19">
         <v>6</v>
       </c>
-      <c r="C517" s="130" t="s">
+      <c r="C517" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E517" s="18">
@@ -23203,7 +23209,7 @@
       <c r="B518" s="19">
         <v>6</v>
       </c>
-      <c r="C518" s="130" t="s">
+      <c r="C518" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E518" s="18">
@@ -23226,7 +23232,7 @@
       <c r="B519" s="19">
         <v>6</v>
       </c>
-      <c r="C519" s="130" t="s">
+      <c r="C519" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E519" s="18">
@@ -23249,7 +23255,7 @@
       <c r="B520" s="19">
         <v>6</v>
       </c>
-      <c r="C520" s="130" t="s">
+      <c r="C520" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E520" s="18">
@@ -23295,7 +23301,7 @@
       <c r="B522" s="19">
         <v>6</v>
       </c>
-      <c r="C522" s="130" t="s">
+      <c r="C522" s="129" t="s">
         <v>277</v>
       </c>
       <c r="E522" s="111">
@@ -23318,7 +23324,7 @@
       <c r="B523" s="19">
         <v>6</v>
       </c>
-      <c r="C523" s="130" t="s">
+      <c r="C523" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E523" s="111">
@@ -23341,7 +23347,7 @@
       <c r="B524" s="19">
         <v>6</v>
       </c>
-      <c r="C524" s="130" t="s">
+      <c r="C524" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E524" s="111">
@@ -23364,7 +23370,7 @@
       <c r="B525" s="19">
         <v>6</v>
       </c>
-      <c r="C525" s="130" t="s">
+      <c r="C525" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E525" s="111">
@@ -23387,7 +23393,7 @@
       <c r="B526" s="39">
         <v>3</v>
       </c>
-      <c r="C526" s="130" t="s">
+      <c r="C526" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E526" s="111">
@@ -23410,7 +23416,7 @@
       <c r="B527" s="39">
         <v>1</v>
       </c>
-      <c r="C527" s="130" t="s">
+      <c r="C527" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E527" s="18">
@@ -23433,7 +23439,7 @@
       <c r="B528" s="39">
         <v>1</v>
       </c>
-      <c r="C528" s="130" t="s">
+      <c r="C528" s="129" t="s">
         <v>480</v>
       </c>
       <c r="E528" s="18">
@@ -24192,7 +24198,7 @@
       <c r="B561" s="39">
         <v>3</v>
       </c>
-      <c r="C561" s="130" t="s">
+      <c r="C561" s="129" t="s">
         <v>478</v>
       </c>
       <c r="E561" s="111">
@@ -24218,7 +24224,7 @@
       <c r="C562" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D562" s="52" t="s">
+      <c r="D562" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E562" s="111">
@@ -24241,7 +24247,7 @@
       <c r="B563" s="39">
         <v>5</v>
       </c>
-      <c r="C563" s="130" t="s">
+      <c r="C563" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E563" s="111">
@@ -24262,12 +24268,12 @@
         <v>267</v>
       </c>
       <c r="B564" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C564" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D564" s="52" t="s">
+      <c r="D564" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E564" s="111">
@@ -24290,7 +24296,7 @@
       <c r="B565" s="19">
         <v>6</v>
       </c>
-      <c r="C565" s="130" t="s">
+      <c r="C565" s="129" t="s">
         <v>275</v>
       </c>
       <c r="E565" s="111">
@@ -24313,7 +24319,7 @@
       <c r="B566" s="19">
         <v>6</v>
       </c>
-      <c r="C566" s="130" t="s">
+      <c r="C566" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E566" s="111">
@@ -24336,7 +24342,7 @@
       <c r="B567" s="39">
         <v>2</v>
       </c>
-      <c r="C567" s="130" t="s">
+      <c r="C567" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E567" s="111">
@@ -24359,7 +24365,7 @@
       <c r="B568" s="19">
         <v>6</v>
       </c>
-      <c r="C568" s="130" t="s">
+      <c r="C568" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E568" s="111">
@@ -24681,7 +24687,7 @@
       <c r="B582" s="19">
         <v>6</v>
       </c>
-      <c r="C582" s="130" t="s">
+      <c r="C582" s="129" t="s">
         <v>270</v>
       </c>
       <c r="E582" s="111">
@@ -24727,7 +24733,7 @@
       <c r="B584" s="39">
         <v>5</v>
       </c>
-      <c r="C584" s="130" t="s">
+      <c r="C584" s="129" t="s">
         <v>278</v>
       </c>
       <c r="E584" s="111">
@@ -24750,7 +24756,7 @@
       <c r="B585" s="19">
         <v>6</v>
       </c>
-      <c r="C585" s="130" t="s">
+      <c r="C585" s="129" t="s">
         <v>272</v>
       </c>
       <c r="E585" s="111">
@@ -24773,7 +24779,7 @@
       <c r="B586" s="39">
         <v>2</v>
       </c>
-      <c r="C586" s="130" t="s">
+      <c r="C586" s="129" t="s">
         <v>479</v>
       </c>
       <c r="E586" s="111">
@@ -24796,7 +24802,7 @@
       <c r="B587" s="19">
         <v>6</v>
       </c>
-      <c r="C587" s="130" t="s">
+      <c r="C587" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E587" s="111">
@@ -24937,7 +24943,7 @@
       <c r="C593" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D593" s="52" t="s">
+      <c r="D593" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E593" s="111">
@@ -25193,7 +25199,7 @@
       <c r="C604" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D604" s="52" t="s">
+      <c r="D604" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E604" s="111">
@@ -25357,7 +25363,7 @@
       <c r="C611" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D611" s="52" t="s">
+      <c r="D611" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E611" s="111">
@@ -25383,7 +25389,7 @@
       <c r="C612" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D612" s="52" t="s">
+      <c r="D612" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E612" s="18">
@@ -25409,7 +25415,7 @@
       <c r="C613" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D613" s="52" t="s">
+      <c r="D613" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E613" s="111">
@@ -25455,7 +25461,7 @@
       <c r="B615" s="19">
         <v>6</v>
       </c>
-      <c r="C615" s="130" t="s">
+      <c r="C615" s="129" t="s">
         <v>274</v>
       </c>
       <c r="E615" s="111">
@@ -25570,7 +25576,7 @@
       <c r="B620" s="19">
         <v>6</v>
       </c>
-      <c r="C620" s="130" t="s">
+      <c r="C620" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E620" s="111">
@@ -25639,7 +25645,7 @@
       <c r="B623" s="19">
         <v>6</v>
       </c>
-      <c r="C623" s="130" t="s">
+      <c r="C623" s="129" t="s">
         <v>271</v>
       </c>
       <c r="E623" s="111">
@@ -25660,12 +25666,12 @@
         <v>267</v>
       </c>
       <c r="B624" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C624" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D624" s="52" t="s">
+      <c r="D624" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E624" s="111">
@@ -25737,7 +25743,7 @@
       <c r="C627" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D627" s="52" t="s">
+      <c r="D627" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E627" s="111">
@@ -25806,7 +25812,7 @@
       <c r="B630" s="19">
         <v>6</v>
       </c>
-      <c r="C630" s="129" t="s">
+      <c r="C630" s="128" t="s">
         <v>274</v>
       </c>
       <c r="E630" s="111">
@@ -25855,7 +25861,7 @@
       <c r="C632" s="39" t="s">
         <v>270</v>
       </c>
-      <c r="D632" s="52" t="s">
+      <c r="D632" s="38" t="s">
         <v>1886</v>
       </c>
       <c r="E632" s="18">
@@ -25904,7 +25910,7 @@
       <c r="C634" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D634" s="52" t="s">
+      <c r="D634" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E634" s="111">
@@ -25948,12 +25954,12 @@
         <v>267</v>
       </c>
       <c r="B636" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C636" s="39" t="s">
         <v>276</v>
       </c>
-      <c r="D636" s="52" t="s">
+      <c r="D636" s="38" t="s">
         <v>1902</v>
       </c>
       <c r="E636" s="111">
@@ -25979,7 +25985,7 @@
       <c r="C637" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D637" s="52"/>
+      <c r="D637" s="38"/>
       <c r="E637" s="111">
         <v>317</v>
       </c>
@@ -26003,7 +26009,7 @@
       <c r="C638" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D638" s="52" t="s">
+      <c r="D638" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E638" s="111">
@@ -26052,7 +26058,7 @@
       <c r="C640" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D640" s="52" t="s">
+      <c r="D640" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E640" s="111">
@@ -26124,7 +26130,7 @@
       <c r="C643" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D643" s="52" t="s">
+      <c r="D643" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E643" s="18">
@@ -26173,7 +26179,7 @@
       <c r="C645" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="D645" s="52" t="s">
+      <c r="D645" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E645" s="111">
@@ -26222,7 +26228,7 @@
       <c r="C647" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="D647" s="52" t="s">
+      <c r="D647" s="38" t="s">
         <v>1888</v>
       </c>
       <c r="E647" s="18">
@@ -26248,7 +26254,7 @@
       <c r="C648" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="D648" s="52" t="s">
+      <c r="D648" s="38" t="s">
         <v>1887</v>
       </c>
       <c r="E648" s="111">
@@ -26274,7 +26280,7 @@
       <c r="C649" s="39" t="s">
         <v>274</v>
       </c>
-      <c r="D649" s="52" t="s">
+      <c r="D649" s="38" t="s">
         <v>1900</v>
       </c>
       <c r="E649" s="18">
@@ -26323,7 +26329,7 @@
       <c r="C651" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="D651" s="52" t="s">
+      <c r="D651" s="38" t="s">
         <v>1901</v>
       </c>
       <c r="E651" s="111">

</xml_diff>